<commit_message>
first german v2 frictionless function
</commit_message>
<xml_diff>
--- a/3_Projects_and_Labs/2_MS_Excel/1_ExcelIsfu_lab/3_CountingAddingWithCriteria.xlsx
+++ b/3_Projects_and_Labs/2_MS_Excel/1_ExcelIsfu_lab/3_CountingAddingWithCriteria.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\birun\Synk\Project_LIFE\Rb_Excel_Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA82288B-B70E-44B8-AF6F-D2CFD2D68E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A799631-AC33-4AE4-89DB-50917E2681A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{6FD467D4-AAA8-448C-9138-D44A67AF1172}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="3" activeTab="9" xr2:uid="{6FD467D4-AAA8-448C-9138-D44A67AF1172}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="10" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="HW(3an)" sheetId="9" r:id="rId10"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'HW(1)'!$A$4:$K$13</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'HW(1an)'!$A$4:$K$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="60">
   <si>
     <t>Sale Rep Criteria:</t>
   </si>
@@ -245,6 +246,9 @@
   </si>
   <si>
     <t>Office 2016 Video #15</t>
+  </si>
+  <si>
+    <t>In cell F5 count how many numbers there are in the range C4:C12. In cell G5 count how many words there are in the range B4:B12. In cell H5 add the sales numbers from the range C4:C12. In cells G11 and G13 use the COUNTIFS function to count with one condition/criteria. In cells H11 and H13 use the SUMIFS function to add with one condition/criteria.</t>
   </si>
 </sst>
 </file>
@@ -361,7 +365,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -419,6 +423,53 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -559,12 +610,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -614,8 +672,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="10" fontId="1" fillId="17" borderId="1" xfId="9" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="10">
+    <cellStyle name="40% - Accent1" xfId="4" builtinId="31"/>
+    <cellStyle name="40% - Accent3" xfId="6" builtinId="39"/>
+    <cellStyle name="40% - Accent4" xfId="8" builtinId="43"/>
+    <cellStyle name="40% - Accent6" xfId="9" builtinId="51"/>
+    <cellStyle name="60% - Accent1" xfId="5" builtinId="32"/>
+    <cellStyle name="60% - Accent3" xfId="7" builtinId="40"/>
+    <cellStyle name="Accent1" xfId="3" builtinId="29"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
@@ -663,6 +736,344 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:strRef>
+          <c:f>'HW(3)'!$A$3</c:f>
+          <c:strCache>
+            <c:ptCount val="1"/>
+            <c:pt idx="0">
+              <c:v>Monday Sales</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="7.3602250923869711E-2"/>
+          <c:y val="0.16913960794988298"/>
+          <c:w val="0.87187729658792656"/>
+          <c:h val="0.7174525222623106"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="tx2">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'HW(3)'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Gigi</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Phil</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Sims</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Tina</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Shelia</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'HW(3)'!$B$6:$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0_);[Red]\("$"#,##0\)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>171</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>207</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>286</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>184</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>272</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-50F3-4142-A044-E12BB101F727}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1986592768"/>
+        <c:axId val="1986591328"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1986592768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1986591328"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1986591328"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1986592768"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="accent4">
+        <a:lumMod val="40000"/>
+        <a:lumOff val="60000"/>
+      </a:schemeClr>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1110,7 +1521,550 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -1674,6 +2628,47 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>302374</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>75189</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60F13493-E63F-0985-F611-CEF32DCD7B26}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -3314,6 +4309,8 @@
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
     <col min="9" max="9" width="14.5546875" customWidth="1"/>
     <col min="11" max="12" width="10.5546875" customWidth="1"/>
   </cols>
@@ -3335,211 +4332,272 @@
       <c r="L1" s="40"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="43" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="41" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="46">
         <v>109</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="46">
         <v>133</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="46">
         <v>378</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="46">
         <v>527</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="46">
         <v>243</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="46">
         <v>190</v>
       </c>
-      <c r="K7">
+      <c r="H7" s="47">
+        <f>SUM(B7:G7)</f>
+        <v>1580</v>
+      </c>
+      <c r="I7" s="48">
+        <f>H7/$K$7</f>
+        <v>0.81025641025641026</v>
+      </c>
+      <c r="K7" s="42">
         <v>1950</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="46">
         <v>188</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="46">
         <v>440</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="46">
         <v>472</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="46">
         <v>172</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="46">
         <v>271</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="46">
         <v>203</v>
       </c>
+      <c r="H8" s="47">
+        <f t="shared" ref="H8:H13" si="0">SUM(B8:G8)</f>
+        <v>1746</v>
+      </c>
+      <c r="I8" s="48">
+        <f t="shared" ref="I8:I13" si="1">H8/$K$7</f>
+        <v>0.89538461538461533</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="46">
         <v>372</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="46">
         <v>122</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="46">
         <v>538</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="46">
         <v>143</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="46">
         <v>386</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="46">
         <v>201</v>
       </c>
+      <c r="H9" s="47">
+        <f t="shared" si="0"/>
+        <v>1762</v>
+      </c>
+      <c r="I9" s="48">
+        <f t="shared" si="1"/>
+        <v>0.90358974358974364</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="46">
         <v>145</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="46">
         <v>293</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="46">
         <v>169</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="46">
         <v>193</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="46">
         <v>325</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="46">
         <v>424</v>
       </c>
+      <c r="H10" s="47">
+        <f t="shared" si="0"/>
+        <v>1549</v>
+      </c>
+      <c r="I10" s="48">
+        <f t="shared" si="1"/>
+        <v>0.7943589743589744</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="46">
         <v>457</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="46">
         <v>313</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="46">
         <v>385</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="46">
         <v>430</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="46">
         <v>374</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="46">
         <v>158</v>
       </c>
+      <c r="H11" s="47">
+        <f t="shared" si="0"/>
+        <v>2117</v>
+      </c>
+      <c r="I11" s="48">
+        <f t="shared" si="1"/>
+        <v>1.0856410256410256</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="46">
         <v>367</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="46">
         <v>458</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="46">
         <v>494</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="46">
         <v>146</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="46">
         <v>429</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="46">
         <v>540</v>
       </c>
+      <c r="H12" s="47">
+        <f t="shared" si="0"/>
+        <v>2434</v>
+      </c>
+      <c r="I12" s="48">
+        <f t="shared" si="1"/>
+        <v>1.2482051282051283</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="46">
         <v>211</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="46">
         <v>197</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="46">
         <v>274</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="46">
         <v>252</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="46">
         <v>318</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="46">
         <v>521</v>
+      </c>
+      <c r="H13" s="47">
+        <f t="shared" si="0"/>
+        <v>1773</v>
+      </c>
+      <c r="I13" s="48">
+        <f t="shared" si="1"/>
+        <v>0.90923076923076918</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LSid&amp;CPage &amp;P of &amp;N&amp;R&amp;A - &amp;F</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -3873,7 +4931,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="38" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -3936,9 +4994,18 @@
       <c r="C5" s="9">
         <v>400</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="8"/>
+      <c r="F5" s="7">
+        <f>COUNT(C4:C12)</f>
+        <v>9</v>
+      </c>
+      <c r="G5" s="7">
+        <f>COUNTA(B4:B12)</f>
+        <v>9</v>
+      </c>
+      <c r="H5" s="8">
+        <f>SUM(C4:C12)</f>
+        <v>5900</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
@@ -4038,8 +5105,14 @@
       <c r="F11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="8"/>
+      <c r="G11" s="7">
+        <f>COUNTIF(B4:B12,F11)</f>
+        <v>4</v>
+      </c>
+      <c r="H11" s="8">
+        <f>SUMIFS(C4:C12,B4:B12,F11)</f>
+        <v>2800</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
@@ -4065,8 +5138,14 @@
       <c r="F13" s="3">
         <v>42456</v>
       </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="8"/>
+      <c r="G13" s="7">
+        <f>COUNTIF(A4:A12,F13)</f>
+        <v>4</v>
+      </c>
+      <c r="H13" s="8">
+        <f>SUMIFS(C4:C12,A4:A12,F13)</f>
+        <v>2600</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4398,5 +5477,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>